<commit_message>
Added different configurations for SRAM blocks
</commit_message>
<xml_diff>
--- a/tcam_specifications.xlsx
+++ b/tcam_specifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\System Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79D89B77-0F4F-4E8D-A2CC-BE9F60C440C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3E01A3-7154-4344-AD4E-D57D289799D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{387C6DB9-B678-4119-9B43-1653EEE54FDC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="27">
   <si>
     <t>Configuration</t>
   </si>
@@ -54,27 +54,83 @@
     <t>tcam_64x28</t>
   </si>
   <si>
-    <t>tcam_64x56</t>
-  </si>
-  <si>
-    <t>66.67 MHz</t>
-  </si>
-  <si>
-    <t>40 MHz</t>
-  </si>
-  <si>
-    <t>4 mm^2</t>
-  </si>
-  <si>
-    <t>9 mm2^2</t>
+    <t>sky130_sram_16byte_1rw_32x4_8</t>
+  </si>
+  <si>
+    <t>125 MHz</t>
+  </si>
+  <si>
+    <t>0.0625 mm^2</t>
+  </si>
+  <si>
+    <t>sky130_sram_32byte_1rw_64x4_8</t>
+  </si>
+  <si>
+    <t>sky130_sram_48byte_1rw_96x4_8</t>
+  </si>
+  <si>
+    <t>sky130_sram_64byte_1rw_128x4_8</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>KLAYOUT XOR</t>
+  </si>
+  <si>
+    <t>sky130_sram_36byte_1rw_72x4_8</t>
+  </si>
+  <si>
+    <t>8.37 mW</t>
+  </si>
+  <si>
+    <t>10.51 mW</t>
+  </si>
+  <si>
+    <t>tcam_32x56</t>
+  </si>
+  <si>
+    <t>0.09 mm^2</t>
+  </si>
+  <si>
+    <t>(2.45 + 2*12.5) = 27.45 mW</t>
+  </si>
+  <si>
+    <t>(8.06 + 4*12.5) = 58.06 mW</t>
+  </si>
+  <si>
+    <t>4.19 mW</t>
+  </si>
+  <si>
+    <t>12.23 mW</t>
+  </si>
+  <si>
+    <t>OpenLane flow ran, antenna pin violators</t>
+  </si>
+  <si>
+    <t>2.56 mm^2</t>
+  </si>
+  <si>
+    <t>16.4 mW</t>
+  </si>
+  <si>
+    <t>1.44 mm^2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -90,10 +146,36 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -102,8 +184,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,63 +506,162 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{090A2AB7-EC37-42BA-B8AA-08CCB3BF07C3}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E5:E9"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>